<commit_message>
Remove unused Qm metadata columns
</commit_message>
<xml_diff>
--- a/data_raw/Qm data.xlsx
+++ b/data_raw/Qm data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W317"/>
+  <dimension ref="A1:T317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -436,9 +436,6 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="23" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -542,21 +539,6 @@
           <t>Qm (ug/g)</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Aged condition</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>Solution- added agent</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -641,9 +623,6 @@
       <c r="T2" t="n">
         <v>339.6</v>
       </c>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -730,9 +709,6 @@
       <c r="T3" t="n">
         <v>199.2</v>
       </c>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -819,9 +795,6 @@
       <c r="T4" t="n">
         <v>234.5</v>
       </c>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -908,13 +881,6 @@
       <c r="T5" t="n">
         <v>2523</v>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Nature: Sludge</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -997,9 +963,6 @@
       <c r="T6" t="n">
         <v>30.5</v>
       </c>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1086,9 +1049,6 @@
       <c r="T7" t="n">
         <v>432</v>
       </c>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1173,13 +1133,6 @@
       <c r="T8" t="n">
         <v>265</v>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1266,9 +1219,6 @@
       <c r="T9" t="n">
         <v>8.279999999999999</v>
       </c>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1355,9 +1305,6 @@
       <c r="T10" t="n">
         <v>8.720000000000002</v>
       </c>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1444,9 +1391,6 @@
       <c r="T11" t="n">
         <v>6.289999999999999</v>
       </c>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1533,9 +1477,6 @@
       <c r="T12" t="n">
         <v>41</v>
       </c>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1620,13 +1561,6 @@
       <c r="T13" t="n">
         <v>79.40000000000001</v>
       </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1713,9 +1647,6 @@
       <c r="T14" t="n">
         <v>2840</v>
       </c>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1802,17 +1733,6 @@
       <c r="T15" t="n">
         <v>11830</v>
       </c>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>HA</t>
-        </is>
-      </c>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>HA 20 mg/L</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1899,17 +1819,6 @@
       <c r="T16" t="n">
         <v>11350</v>
       </c>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>HA</t>
-        </is>
-      </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>HA 40 mg/L</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1996,17 +1905,6 @@
       <c r="T17" t="n">
         <v>9420</v>
       </c>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>HA</t>
-        </is>
-      </c>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>HA 60 mg/L</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2093,17 +1991,6 @@
       <c r="T18" t="n">
         <v>11030</v>
       </c>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>FA</t>
-        </is>
-      </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>FA 20 mg/L</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2190,17 +2077,6 @@
       <c r="T19" t="n">
         <v>10380</v>
       </c>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>FA</t>
-        </is>
-      </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>FA 40 mg/L</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2287,17 +2163,6 @@
       <c r="T20" t="n">
         <v>8410</v>
       </c>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>FA</t>
-        </is>
-      </c>
-      <c r="W20" t="inlineStr">
-        <is>
-          <t>FA 60 mg/L</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2382,9 +2247,6 @@
       <c r="T21" t="n">
         <v>36.63</v>
       </c>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2469,9 +2331,6 @@
       <c r="T22" t="n">
         <v>36.1</v>
       </c>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2556,9 +2415,6 @@
       <c r="T23" t="n">
         <v>40.49</v>
       </c>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2643,9 +2499,6 @@
       <c r="T24" t="n">
         <v>53.48</v>
       </c>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2730,9 +2583,6 @@
       <c r="T25" t="n">
         <v>160</v>
       </c>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2817,13 +2667,6 @@
       <c r="T26" t="n">
         <v>183</v>
       </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>Lab: 1 month UV</t>
-        </is>
-      </c>
-      <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2908,13 +2751,6 @@
       <c r="T27" t="n">
         <v>203</v>
       </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>Lab: 2 month UV</t>
-        </is>
-      </c>
-      <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2999,13 +2835,6 @@
       <c r="T28" t="n">
         <v>202</v>
       </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>Lab: 3 month UV</t>
-        </is>
-      </c>
-      <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3090,9 +2919,6 @@
       <c r="T29" t="n">
         <v>210</v>
       </c>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3177,13 +3003,6 @@
       <c r="T30" t="n">
         <v>171</v>
       </c>
-      <c r="U30" t="inlineStr">
-        <is>
-          <t>Lab: 1 month UV</t>
-        </is>
-      </c>
-      <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3268,13 +3087,6 @@
       <c r="T31" t="n">
         <v>162</v>
       </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>Lab: 2 month UV</t>
-        </is>
-      </c>
-      <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3359,13 +3171,6 @@
       <c r="T32" t="n">
         <v>173</v>
       </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>Lab: 3 month UV</t>
-        </is>
-      </c>
-      <c r="V32" t="inlineStr"/>
-      <c r="W32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3450,9 +3255,6 @@
       <c r="T33" t="n">
         <v>105</v>
       </c>
-      <c r="U33" t="inlineStr"/>
-      <c r="V33" t="inlineStr"/>
-      <c r="W33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3537,13 +3339,6 @@
       <c r="T34" t="n">
         <v>133</v>
       </c>
-      <c r="U34" t="inlineStr">
-        <is>
-          <t>Lab: 1 month UV</t>
-        </is>
-      </c>
-      <c r="V34" t="inlineStr"/>
-      <c r="W34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3628,13 +3423,6 @@
       <c r="T35" t="n">
         <v>157</v>
       </c>
-      <c r="U35" t="inlineStr">
-        <is>
-          <t>Lab: 2 month UV</t>
-        </is>
-      </c>
-      <c r="V35" t="inlineStr"/>
-      <c r="W35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3719,13 +3507,6 @@
       <c r="T36" t="n">
         <v>175</v>
       </c>
-      <c r="U36" t="inlineStr">
-        <is>
-          <t>Lab: 3 month UV</t>
-        </is>
-      </c>
-      <c r="V36" t="inlineStr"/>
-      <c r="W36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3810,9 +3591,6 @@
       <c r="T37" t="n">
         <v>125</v>
       </c>
-      <c r="U37" t="inlineStr"/>
-      <c r="V37" t="inlineStr"/>
-      <c r="W37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3897,13 +3675,6 @@
       <c r="T38" t="n">
         <v>140</v>
       </c>
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>Lab: 1 month UV</t>
-        </is>
-      </c>
-      <c r="V38" t="inlineStr"/>
-      <c r="W38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3988,13 +3759,6 @@
       <c r="T39" t="n">
         <v>143</v>
       </c>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>Lab: 2 month UV</t>
-        </is>
-      </c>
-      <c r="V39" t="inlineStr"/>
-      <c r="W39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4079,13 +3843,6 @@
       <c r="T40" t="n">
         <v>196</v>
       </c>
-      <c r="U40" t="inlineStr">
-        <is>
-          <t>Lab: 3 month UV</t>
-        </is>
-      </c>
-      <c r="V40" t="inlineStr"/>
-      <c r="W40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4170,9 +3927,6 @@
       <c r="T41" t="n">
         <v>78.09999999999999</v>
       </c>
-      <c r="U41" t="inlineStr"/>
-      <c r="V41" t="inlineStr"/>
-      <c r="W41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4257,13 +4011,6 @@
       <c r="T42" t="n">
         <v>128</v>
       </c>
-      <c r="U42" t="inlineStr">
-        <is>
-          <t>Lab: 1 month UV</t>
-        </is>
-      </c>
-      <c r="V42" t="inlineStr"/>
-      <c r="W42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4348,13 +4095,6 @@
       <c r="T43" t="n">
         <v>158</v>
       </c>
-      <c r="U43" t="inlineStr">
-        <is>
-          <t>Lab: 2 month UV</t>
-        </is>
-      </c>
-      <c r="V43" t="inlineStr"/>
-      <c r="W43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4439,13 +4179,6 @@
       <c r="T44" t="n">
         <v>183</v>
       </c>
-      <c r="U44" t="inlineStr">
-        <is>
-          <t>Lab: 3 month UV</t>
-        </is>
-      </c>
-      <c r="V44" t="inlineStr"/>
-      <c r="W44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4530,13 +4263,6 @@
       <c r="T45" t="n">
         <v>199</v>
       </c>
-      <c r="U45" t="inlineStr">
-        <is>
-          <t>Lab: 3 month-pure water</t>
-        </is>
-      </c>
-      <c r="V45" t="inlineStr"/>
-      <c r="W45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4621,13 +4347,6 @@
       <c r="T46" t="n">
         <v>199</v>
       </c>
-      <c r="U46" t="inlineStr">
-        <is>
-          <t>Lab: 3 month-sea water</t>
-        </is>
-      </c>
-      <c r="V46" t="inlineStr"/>
-      <c r="W46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4712,13 +4431,6 @@
       <c r="T47" t="n">
         <v>202</v>
       </c>
-      <c r="U47" t="inlineStr">
-        <is>
-          <t>Lab: 3 month-air</t>
-        </is>
-      </c>
-      <c r="V47" t="inlineStr"/>
-      <c r="W47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4803,13 +4515,6 @@
       <c r="T48" t="n">
         <v>176</v>
       </c>
-      <c r="U48" t="inlineStr">
-        <is>
-          <t>Lab: 3 month-pure water</t>
-        </is>
-      </c>
-      <c r="V48" t="inlineStr"/>
-      <c r="W48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4894,13 +4599,6 @@
       <c r="T49" t="n">
         <v>170</v>
       </c>
-      <c r="U49" t="inlineStr">
-        <is>
-          <t>Lab: 3 month-sea water</t>
-        </is>
-      </c>
-      <c r="V49" t="inlineStr"/>
-      <c r="W49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4985,13 +4683,6 @@
       <c r="T50" t="n">
         <v>173</v>
       </c>
-      <c r="U50" t="inlineStr">
-        <is>
-          <t>Lab: 3 month-air</t>
-        </is>
-      </c>
-      <c r="V50" t="inlineStr"/>
-      <c r="W50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5076,13 +4767,6 @@
       <c r="T51" t="n">
         <v>168</v>
       </c>
-      <c r="U51" t="inlineStr">
-        <is>
-          <t>Lab: 3 month-pure water</t>
-        </is>
-      </c>
-      <c r="V51" t="inlineStr"/>
-      <c r="W51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5167,13 +4851,6 @@
       <c r="T52" t="n">
         <v>161</v>
       </c>
-      <c r="U52" t="inlineStr">
-        <is>
-          <t>Lab: 3 month-sea water</t>
-        </is>
-      </c>
-      <c r="V52" t="inlineStr"/>
-      <c r="W52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5258,13 +4935,6 @@
       <c r="T53" t="n">
         <v>175</v>
       </c>
-      <c r="U53" t="inlineStr">
-        <is>
-          <t>Lab: 3 month-air</t>
-        </is>
-      </c>
-      <c r="V53" t="inlineStr"/>
-      <c r="W53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5349,13 +5019,6 @@
       <c r="T54" t="n">
         <v>259</v>
       </c>
-      <c r="U54" t="inlineStr">
-        <is>
-          <t>Lab: 3 month-pure water</t>
-        </is>
-      </c>
-      <c r="V54" t="inlineStr"/>
-      <c r="W54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5440,13 +5103,6 @@
       <c r="T55" t="n">
         <v>211</v>
       </c>
-      <c r="U55" t="inlineStr">
-        <is>
-          <t>Lab: 3 month-sea water</t>
-        </is>
-      </c>
-      <c r="V55" t="inlineStr"/>
-      <c r="W55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5531,13 +5187,6 @@
       <c r="T56" t="n">
         <v>196</v>
       </c>
-      <c r="U56" t="inlineStr">
-        <is>
-          <t>Lab: 3 month-air</t>
-        </is>
-      </c>
-      <c r="V56" t="inlineStr"/>
-      <c r="W56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5622,13 +5271,6 @@
       <c r="T57" t="n">
         <v>312</v>
       </c>
-      <c r="U57" t="inlineStr">
-        <is>
-          <t>Lab: 3 month-pure water</t>
-        </is>
-      </c>
-      <c r="V57" t="inlineStr"/>
-      <c r="W57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5713,13 +5355,6 @@
       <c r="T58" t="n">
         <v>236</v>
       </c>
-      <c r="U58" t="inlineStr">
-        <is>
-          <t>Lab: 3 month-sea water</t>
-        </is>
-      </c>
-      <c r="V58" t="inlineStr"/>
-      <c r="W58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5804,13 +5439,6 @@
       <c r="T59" t="n">
         <v>183</v>
       </c>
-      <c r="U59" t="inlineStr">
-        <is>
-          <t>Lab: 3 month-air</t>
-        </is>
-      </c>
-      <c r="V59" t="inlineStr"/>
-      <c r="W59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5897,13 +5525,6 @@
       <c r="T60" t="n">
         <v>463.7</v>
       </c>
-      <c r="U60" t="inlineStr">
-        <is>
-          <t>Nature: coastal aquaculture</t>
-        </is>
-      </c>
-      <c r="V60" t="inlineStr"/>
-      <c r="W60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5990,13 +5611,6 @@
       <c r="T61" t="n">
         <v>1031.5</v>
       </c>
-      <c r="U61" t="inlineStr">
-        <is>
-          <t>Nature: coastal aquaculture</t>
-        </is>
-      </c>
-      <c r="V61" t="inlineStr"/>
-      <c r="W61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6081,17 +5695,6 @@
       <c r="T62" t="n">
         <v>335.48</v>
       </c>
-      <c r="U62" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V62" t="inlineStr"/>
-      <c r="W62" t="inlineStr">
-        <is>
-          <t>The adsorption behavior of metals</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -6176,13 +5779,6 @@
       <c r="T63" t="n">
         <v>211.03</v>
       </c>
-      <c r="U63" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V63" t="inlineStr"/>
-      <c r="W63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6267,13 +5863,6 @@
       <c r="T64" t="n">
         <v>318.42</v>
       </c>
-      <c r="U64" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V64" t="inlineStr"/>
-      <c r="W64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6358,9 +5947,6 @@
       <c r="T65" t="n">
         <v>237.5</v>
       </c>
-      <c r="U65" t="inlineStr"/>
-      <c r="V65" t="inlineStr"/>
-      <c r="W65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -6445,21 +6031,6 @@
       <c r="T66" t="n">
         <v>762.2</v>
       </c>
-      <c r="U66" t="inlineStr">
-        <is>
-          <t>Lab: Wastewater, 20d</t>
-        </is>
-      </c>
-      <c r="V66" t="inlineStr">
-        <is>
-          <t>TC</t>
-        </is>
-      </c>
-      <c r="W66" t="inlineStr">
-        <is>
-          <t>PE+5 mg/L TC</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -6544,9 +6115,6 @@
       <c r="T67" t="n">
         <v>777.1799999999999</v>
       </c>
-      <c r="U67" t="inlineStr"/>
-      <c r="V67" t="inlineStr"/>
-      <c r="W67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -6631,13 +6199,6 @@
       <c r="T68" t="n">
         <v>1566.94</v>
       </c>
-      <c r="U68" t="inlineStr">
-        <is>
-          <t>Lab: UV seawater</t>
-        </is>
-      </c>
-      <c r="V68" t="inlineStr"/>
-      <c r="W68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -6722,9 +6283,6 @@
       <c r="T69" t="n">
         <v>715.99</v>
       </c>
-      <c r="U69" t="inlineStr"/>
-      <c r="V69" t="inlineStr"/>
-      <c r="W69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6809,13 +6367,6 @@
       <c r="T70" t="n">
         <v>1282.35</v>
       </c>
-      <c r="U70" t="inlineStr">
-        <is>
-          <t>Lab: UV seawater</t>
-        </is>
-      </c>
-      <c r="V70" t="inlineStr"/>
-      <c r="W70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6900,9 +6451,6 @@
       <c r="T71" t="n">
         <v>1369.33</v>
       </c>
-      <c r="U71" t="inlineStr"/>
-      <c r="V71" t="inlineStr"/>
-      <c r="W71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6987,13 +6535,6 @@
       <c r="T72" t="n">
         <v>3903.1</v>
       </c>
-      <c r="U72" t="inlineStr">
-        <is>
-          <t>Lab: UV seawater</t>
-        </is>
-      </c>
-      <c r="V72" t="inlineStr"/>
-      <c r="W72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -7078,9 +6619,6 @@
       <c r="T73" t="n">
         <v>1371.13</v>
       </c>
-      <c r="U73" t="inlineStr"/>
-      <c r="V73" t="inlineStr"/>
-      <c r="W73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7165,13 +6703,6 @@
       <c r="T74" t="n">
         <v>2366.53</v>
       </c>
-      <c r="U74" t="inlineStr">
-        <is>
-          <t>Lab: UV seawater</t>
-        </is>
-      </c>
-      <c r="V74" t="inlineStr"/>
-      <c r="W74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7258,9 +6789,6 @@
       <c r="T75" t="n">
         <v>339.6</v>
       </c>
-      <c r="U75" t="inlineStr"/>
-      <c r="V75" t="inlineStr"/>
-      <c r="W75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -7347,13 +6875,6 @@
       <c r="T76" t="n">
         <v>2130</v>
       </c>
-      <c r="U76" t="inlineStr">
-        <is>
-          <t>Lab: Wastewater pipeline</t>
-        </is>
-      </c>
-      <c r="V76" t="inlineStr"/>
-      <c r="W76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -7440,13 +6961,6 @@
       <c r="T77" t="n">
         <v>126.5</v>
       </c>
-      <c r="U77" t="inlineStr">
-        <is>
-          <t>Lab: Grit tank</t>
-        </is>
-      </c>
-      <c r="V77" t="inlineStr"/>
-      <c r="W77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -7533,13 +7047,6 @@
       <c r="T78" t="n">
         <v>614.48</v>
       </c>
-      <c r="U78" t="inlineStr">
-        <is>
-          <t>Lab: Aeration tank</t>
-        </is>
-      </c>
-      <c r="V78" t="inlineStr"/>
-      <c r="W78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7626,13 +7133,6 @@
       <c r="T79" t="n">
         <v>57.48</v>
       </c>
-      <c r="U79" t="inlineStr">
-        <is>
-          <t>Lab: Aeration tank</t>
-        </is>
-      </c>
-      <c r="V79" t="inlineStr"/>
-      <c r="W79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -7717,9 +7217,6 @@
       <c r="T80" t="n">
         <v>650.7</v>
       </c>
-      <c r="U80" t="inlineStr"/>
-      <c r="V80" t="inlineStr"/>
-      <c r="W80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -7804,9 +7301,6 @@
       <c r="T81" t="n">
         <v>794.8</v>
       </c>
-      <c r="U81" t="inlineStr"/>
-      <c r="V81" t="inlineStr"/>
-      <c r="W81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7891,9 +7385,6 @@
       <c r="T82" t="n">
         <v>943.2</v>
       </c>
-      <c r="U82" t="inlineStr"/>
-      <c r="V82" t="inlineStr"/>
-      <c r="W82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7976,9 +7467,6 @@
       <c r="T83" t="n">
         <v>613.1</v>
       </c>
-      <c r="U83" t="inlineStr"/>
-      <c r="V83" t="inlineStr"/>
-      <c r="W83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -8061,17 +7549,6 @@
       <c r="T84" t="n">
         <v>1239.72</v>
       </c>
-      <c r="U84" t="inlineStr">
-        <is>
-          <t>Nature: Lake</t>
-        </is>
-      </c>
-      <c r="V84" t="inlineStr"/>
-      <c r="W84" t="inlineStr">
-        <is>
-          <t>PS+biofilm+Nanhu</t>
-        </is>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -8153,17 +7630,6 @@
       </c>
       <c r="T85" t="n">
         <v>1101.41</v>
-      </c>
-      <c r="U85" t="inlineStr">
-        <is>
-          <t>Nature: Lake</t>
-        </is>
-      </c>
-      <c r="V85" t="inlineStr"/>
-      <c r="W85" t="inlineStr">
-        <is>
-          <t>PS+biofilm+Shitoukoumen</t>
-        </is>
       </c>
     </row>
     <row r="86">
@@ -8247,9 +7713,6 @@
       <c r="T86" t="n">
         <v>31.2</v>
       </c>
-      <c r="U86" t="inlineStr"/>
-      <c r="V86" t="inlineStr"/>
-      <c r="W86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -8332,17 +7795,6 @@
       <c r="T87" t="n">
         <v>183</v>
       </c>
-      <c r="U87" t="inlineStr">
-        <is>
-          <t>Lab: air incubating</t>
-        </is>
-      </c>
-      <c r="V87" t="inlineStr"/>
-      <c r="W87" t="inlineStr">
-        <is>
-          <t>Aged MP (A-PE-MPs)</t>
-        </is>
-      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -8425,17 +7877,6 @@
       <c r="T88" t="n">
         <v>108</v>
       </c>
-      <c r="U88" t="inlineStr">
-        <is>
-          <t>Lab: water incubating</t>
-        </is>
-      </c>
-      <c r="V88" t="inlineStr"/>
-      <c r="W88" t="inlineStr">
-        <is>
-          <t>Aged MP (W-PE-MPs)</t>
-        </is>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -8518,17 +7959,6 @@
       <c r="T89" t="n">
         <v>318</v>
       </c>
-      <c r="U89" t="inlineStr">
-        <is>
-          <t>Lab: soil incubating</t>
-        </is>
-      </c>
-      <c r="V89" t="inlineStr"/>
-      <c r="W89" t="inlineStr">
-        <is>
-          <t>Aged MP (S-PE-MPs)</t>
-        </is>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -8611,13 +8041,6 @@
       <c r="T90" t="n">
         <v>42.6</v>
       </c>
-      <c r="U90" t="inlineStr"/>
-      <c r="V90" t="inlineStr">
-        <is>
-          <t>TC</t>
-        </is>
-      </c>
-      <c r="W90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -8700,17 +8123,6 @@
       <c r="T91" t="n">
         <v>412</v>
       </c>
-      <c r="U91" t="inlineStr">
-        <is>
-          <t>Lab: air incubating</t>
-        </is>
-      </c>
-      <c r="V91" t="inlineStr">
-        <is>
-          <t>TC</t>
-        </is>
-      </c>
-      <c r="W91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -8793,17 +8205,6 @@
       <c r="T92" t="n">
         <v>120</v>
       </c>
-      <c r="U92" t="inlineStr">
-        <is>
-          <t>Lab: water incubating</t>
-        </is>
-      </c>
-      <c r="V92" t="inlineStr">
-        <is>
-          <t>TC</t>
-        </is>
-      </c>
-      <c r="W92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -8886,17 +8287,6 @@
       <c r="T93" t="n">
         <v>210</v>
       </c>
-      <c r="U93" t="inlineStr">
-        <is>
-          <t>Lab: soil incubating</t>
-        </is>
-      </c>
-      <c r="V93" t="inlineStr">
-        <is>
-          <t>TC</t>
-        </is>
-      </c>
-      <c r="W93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -8979,9 +8369,6 @@
       <c r="T94" t="n">
         <v>454</v>
       </c>
-      <c r="U94" t="inlineStr"/>
-      <c r="V94" t="inlineStr"/>
-      <c r="W94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -9064,13 +8451,6 @@
       <c r="T95" t="n">
         <v>521</v>
       </c>
-      <c r="U95" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V95" t="inlineStr"/>
-      <c r="W95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -9153,13 +8533,6 @@
       <c r="T96" t="n">
         <v>613</v>
       </c>
-      <c r="U96" t="inlineStr"/>
-      <c r="V96" t="inlineStr">
-        <is>
-          <t>OTC</t>
-        </is>
-      </c>
-      <c r="W96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -9242,17 +8615,6 @@
       <c r="T97" t="n">
         <v>576</v>
       </c>
-      <c r="U97" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V97" t="inlineStr">
-        <is>
-          <t>OTC</t>
-        </is>
-      </c>
-      <c r="W97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -9335,13 +8697,6 @@
       <c r="T98" t="n">
         <v>655.6999999999999</v>
       </c>
-      <c r="U98" t="inlineStr"/>
-      <c r="V98" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hexabromocyclododecane </t>
-        </is>
-      </c>
-      <c r="W98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -9424,13 +8779,6 @@
       <c r="T99" t="n">
         <v>784.5999999999999</v>
       </c>
-      <c r="U99" t="inlineStr"/>
-      <c r="V99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hexabromocyclododecane </t>
-        </is>
-      </c>
-      <c r="W99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -9513,13 +8861,6 @@
       <c r="T100" t="n">
         <v>926.4</v>
       </c>
-      <c r="U100" t="inlineStr"/>
-      <c r="V100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">hexabromocyclododecane </t>
-        </is>
-      </c>
-      <c r="W100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -9602,17 +8943,6 @@
       <c r="T101" t="n">
         <v>463.8</v>
       </c>
-      <c r="U101" t="inlineStr">
-        <is>
-          <t>Lab: Alkaline aging</t>
-        </is>
-      </c>
-      <c r="V101" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HA </t>
-        </is>
-      </c>
-      <c r="W101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -9695,17 +9025,6 @@
       <c r="T102" t="n">
         <v>817.2</v>
       </c>
-      <c r="U102" t="inlineStr">
-        <is>
-          <t>Lab: Alkaline aging</t>
-        </is>
-      </c>
-      <c r="V102" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HA </t>
-        </is>
-      </c>
-      <c r="W102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -9788,17 +9107,6 @@
       <c r="T103" t="n">
         <v>970.7</v>
       </c>
-      <c r="U103" t="inlineStr">
-        <is>
-          <t>Lab: Alkaline aging</t>
-        </is>
-      </c>
-      <c r="V103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HA </t>
-        </is>
-      </c>
-      <c r="W103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -9881,9 +9189,6 @@
       <c r="T104" t="n">
         <v>239.9</v>
       </c>
-      <c r="U104" t="inlineStr"/>
-      <c r="V104" t="inlineStr"/>
-      <c r="W104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -9966,17 +9271,6 @@
       <c r="T105" t="n">
         <v>481.7</v>
       </c>
-      <c r="U105" t="inlineStr"/>
-      <c r="V105" t="inlineStr">
-        <is>
-          <t>CTAB</t>
-        </is>
-      </c>
-      <c r="W105" t="inlineStr">
-        <is>
-          <t>PE-CTAB</t>
-        </is>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -10059,17 +9353,6 @@
       <c r="T106" t="n">
         <v>1031.2</v>
       </c>
-      <c r="U106" t="inlineStr"/>
-      <c r="V106" t="inlineStr">
-        <is>
-          <t>SDBS</t>
-        </is>
-      </c>
-      <c r="W106" t="inlineStr">
-        <is>
-          <t>PE-SDBS</t>
-        </is>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -10152,9 +9435,6 @@
       <c r="T107" t="n">
         <v>1890.4</v>
       </c>
-      <c r="U107" t="inlineStr"/>
-      <c r="V107" t="inlineStr"/>
-      <c r="W107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -10237,17 +9517,6 @@
       <c r="T108" t="n">
         <v>1375.1</v>
       </c>
-      <c r="U108" t="inlineStr"/>
-      <c r="V108" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CTAB </t>
-        </is>
-      </c>
-      <c r="W108" t="inlineStr">
-        <is>
-          <t>PP-CTAB</t>
-        </is>
-      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -10330,17 +9599,6 @@
       <c r="T109" t="n">
         <v>2513.2</v>
       </c>
-      <c r="U109" t="inlineStr"/>
-      <c r="V109" t="inlineStr">
-        <is>
-          <t>SDBS</t>
-        </is>
-      </c>
-      <c r="W109" t="inlineStr">
-        <is>
-          <t>PP-SDBS</t>
-        </is>
-      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -10423,13 +9681,6 @@
       <c r="T110" t="n">
         <v>3474</v>
       </c>
-      <c r="U110" t="inlineStr"/>
-      <c r="V110" t="inlineStr"/>
-      <c r="W110" t="inlineStr">
-        <is>
-          <t>Comparing the influence….</t>
-        </is>
-      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -10512,17 +9763,6 @@
       <c r="T111" t="n">
         <v>917</v>
       </c>
-      <c r="U111" t="inlineStr"/>
-      <c r="V111" t="inlineStr">
-        <is>
-          <t>FA</t>
-        </is>
-      </c>
-      <c r="W111" t="inlineStr">
-        <is>
-          <t>PS+FA10</t>
-        </is>
-      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -10605,17 +9845,6 @@
       <c r="T112" t="n">
         <v>704</v>
       </c>
-      <c r="U112" t="inlineStr"/>
-      <c r="V112" t="inlineStr">
-        <is>
-          <t>FA</t>
-        </is>
-      </c>
-      <c r="W112" t="inlineStr">
-        <is>
-          <t>PS+FA20</t>
-        </is>
-      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -10698,17 +9927,6 @@
       <c r="T113" t="n">
         <v>4527</v>
       </c>
-      <c r="U113" t="inlineStr"/>
-      <c r="V113" t="inlineStr">
-        <is>
-          <t>TA</t>
-        </is>
-      </c>
-      <c r="W113" t="inlineStr">
-        <is>
-          <t>PS+TA10</t>
-        </is>
-      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -10791,17 +10009,6 @@
       <c r="T114" t="n">
         <v>4901</v>
       </c>
-      <c r="U114" t="inlineStr"/>
-      <c r="V114" t="inlineStr">
-        <is>
-          <t>TA</t>
-        </is>
-      </c>
-      <c r="W114" t="inlineStr">
-        <is>
-          <t>PS+TA20</t>
-        </is>
-      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -10884,17 +10091,6 @@
       <c r="T115" t="n">
         <v>2598</v>
       </c>
-      <c r="U115" t="inlineStr"/>
-      <c r="V115" t="inlineStr">
-        <is>
-          <t>HA</t>
-        </is>
-      </c>
-      <c r="W115" t="inlineStr">
-        <is>
-          <t>PS+HA10</t>
-        </is>
-      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -10977,17 +10173,6 @@
       <c r="T116" t="n">
         <v>1786</v>
       </c>
-      <c r="U116" t="inlineStr"/>
-      <c r="V116" t="inlineStr">
-        <is>
-          <t>HA</t>
-        </is>
-      </c>
-      <c r="W116" t="inlineStr">
-        <is>
-          <t>PS+HA20</t>
-        </is>
-      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -11074,13 +10259,6 @@
       <c r="T117" t="n">
         <v>511</v>
       </c>
-      <c r="U117" t="inlineStr"/>
-      <c r="V117" t="inlineStr"/>
-      <c r="W117" t="inlineStr">
-        <is>
-          <t>Adsorption of lead and cadmium by…</t>
-        </is>
-      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -11167,9 +10345,6 @@
       <c r="T118" t="n">
         <v>775</v>
       </c>
-      <c r="U118" t="inlineStr"/>
-      <c r="V118" t="inlineStr"/>
-      <c r="W118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -11256,9 +10431,6 @@
       <c r="T119" t="n">
         <v>314</v>
       </c>
-      <c r="U119" t="inlineStr"/>
-      <c r="V119" t="inlineStr"/>
-      <c r="W119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -11345,9 +10517,6 @@
       <c r="T120" t="n">
         <v>323</v>
       </c>
-      <c r="U120" t="inlineStr"/>
-      <c r="V120" t="inlineStr"/>
-      <c r="W120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -11434,13 +10603,6 @@
       <c r="T121" t="n">
         <v>64.13</v>
       </c>
-      <c r="U121" t="inlineStr"/>
-      <c r="V121" t="inlineStr"/>
-      <c r="W121" t="inlineStr">
-        <is>
-          <t>Effect of biofilm colonization…</t>
-        </is>
-      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -11527,17 +10689,6 @@
       <c r="T122" t="n">
         <v>647.09</v>
       </c>
-      <c r="U122" t="inlineStr">
-        <is>
-          <t>Lab: wastewater-incubation</t>
-        </is>
-      </c>
-      <c r="V122" t="inlineStr"/>
-      <c r="W122" t="inlineStr">
-        <is>
-          <t>Aged MP (biofilm)</t>
-        </is>
-      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -11623,17 +10774,6 @@
       </c>
       <c r="T123" t="n">
         <v>323.62</v>
-      </c>
-      <c r="U123" t="inlineStr">
-        <is>
-          <t>Lab: wastewater-incubation</t>
-        </is>
-      </c>
-      <c r="V123" t="inlineStr"/>
-      <c r="W123" t="inlineStr">
-        <is>
-          <t>Aged MP (biofilm removed)</t>
-        </is>
       </c>
     </row>
     <row r="124">
@@ -11719,13 +10859,6 @@
       <c r="T124" t="n">
         <v>95.77</v>
       </c>
-      <c r="U124" t="inlineStr"/>
-      <c r="V124" t="inlineStr"/>
-      <c r="W124" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Adsorption behaviour of </t>
-        </is>
-      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -11812,9 +10945,6 @@
       <c r="T125" t="n">
         <v>588.42</v>
       </c>
-      <c r="U125" t="inlineStr"/>
-      <c r="V125" t="inlineStr"/>
-      <c r="W125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -11899,9 +11029,6 @@
       <c r="T126" t="n">
         <v>69.03</v>
       </c>
-      <c r="U126" t="inlineStr"/>
-      <c r="V126" t="inlineStr"/>
-      <c r="W126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -11986,9 +11113,6 @@
       <c r="T127" t="n">
         <v>164.54</v>
       </c>
-      <c r="U127" t="inlineStr"/>
-      <c r="V127" t="inlineStr"/>
-      <c r="W127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -12075,9 +11199,6 @@
       <c r="T128" t="n">
         <v>797.61</v>
       </c>
-      <c r="U128" t="inlineStr"/>
-      <c r="V128" t="inlineStr"/>
-      <c r="W128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -12162,9 +11283,6 @@
       <c r="T129" t="n">
         <v>238.47</v>
       </c>
-      <c r="U129" t="inlineStr"/>
-      <c r="V129" t="inlineStr"/>
-      <c r="W129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -12251,9 +11369,6 @@
       <c r="T130" t="n">
         <v>745.26</v>
       </c>
-      <c r="U130" t="inlineStr"/>
-      <c r="V130" t="inlineStr"/>
-      <c r="W130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -12338,9 +11453,6 @@
       <c r="T131" t="n">
         <v>85.67</v>
       </c>
-      <c r="U131" t="inlineStr"/>
-      <c r="V131" t="inlineStr"/>
-      <c r="W131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -12427,9 +11539,6 @@
       <c r="T132" t="n">
         <v>791.4400000000001</v>
       </c>
-      <c r="U132" t="inlineStr"/>
-      <c r="V132" t="inlineStr"/>
-      <c r="W132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -12514,13 +11623,6 @@
       <c r="T133" t="n">
         <v>715.54</v>
       </c>
-      <c r="U133" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V133" t="inlineStr"/>
-      <c r="W133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -12605,13 +11707,6 @@
       <c r="T134" t="n">
         <v>261.17</v>
       </c>
-      <c r="U134" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V134" t="inlineStr"/>
-      <c r="W134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -12696,13 +11791,6 @@
       <c r="T135" t="n">
         <v>726.75</v>
       </c>
-      <c r="U135" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V135" t="inlineStr"/>
-      <c r="W135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -12787,13 +11875,6 @@
       <c r="T136" t="n">
         <v>330.61</v>
       </c>
-      <c r="U136" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V136" t="inlineStr"/>
-      <c r="W136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -12878,13 +11959,6 @@
       <c r="T137" t="n">
         <v>244.34</v>
       </c>
-      <c r="U137" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V137" t="inlineStr"/>
-      <c r="W137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -12969,13 +12043,6 @@
       <c r="T138" t="n">
         <v>796.66</v>
       </c>
-      <c r="U138" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V138" t="inlineStr"/>
-      <c r="W138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -13058,13 +12125,6 @@
       <c r="T139" t="n">
         <v>33.275</v>
       </c>
-      <c r="U139" t="inlineStr"/>
-      <c r="V139" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HBCD </t>
-        </is>
-      </c>
-      <c r="W139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -13147,13 +12207,6 @@
       <c r="T140" t="n">
         <v>40.111</v>
       </c>
-      <c r="U140" t="inlineStr"/>
-      <c r="V140" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HBCD </t>
-        </is>
-      </c>
-      <c r="W140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -13236,13 +12289,6 @@
       <c r="T141" t="n">
         <v>48.217</v>
       </c>
-      <c r="U141" t="inlineStr"/>
-      <c r="V141" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HBCD </t>
-        </is>
-      </c>
-      <c r="W141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -13325,13 +12371,6 @@
       <c r="T142" t="n">
         <v>15.577</v>
       </c>
-      <c r="U142" t="inlineStr"/>
-      <c r="V142" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HBCD </t>
-        </is>
-      </c>
-      <c r="W142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -13414,13 +12453,6 @@
       <c r="T143" t="n">
         <v>23.213</v>
       </c>
-      <c r="U143" t="inlineStr"/>
-      <c r="V143" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HBCD </t>
-        </is>
-      </c>
-      <c r="W143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -13503,13 +12535,6 @@
       <c r="T144" t="n">
         <v>27.569</v>
       </c>
-      <c r="U144" t="inlineStr"/>
-      <c r="V144" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HBCD </t>
-        </is>
-      </c>
-      <c r="W144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -13592,13 +12617,6 @@
       <c r="T145" t="n">
         <v>9.228</v>
       </c>
-      <c r="U145" t="inlineStr"/>
-      <c r="V145" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HBCD </t>
-        </is>
-      </c>
-      <c r="W145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -13681,13 +12699,6 @@
       <c r="T146" t="n">
         <v>11.724</v>
       </c>
-      <c r="U146" t="inlineStr"/>
-      <c r="V146" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HBCD </t>
-        </is>
-      </c>
-      <c r="W146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -13770,13 +12781,6 @@
       <c r="T147" t="n">
         <v>13.416</v>
       </c>
-      <c r="U147" t="inlineStr"/>
-      <c r="V147" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HBCD </t>
-        </is>
-      </c>
-      <c r="W147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -13861,13 +12865,6 @@
       <c r="T148" t="n">
         <v>9250</v>
       </c>
-      <c r="U148" t="inlineStr"/>
-      <c r="V148" t="inlineStr"/>
-      <c r="W148" t="inlineStr">
-        <is>
-          <t>Investigation of the adsorption</t>
-        </is>
-      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -13952,17 +12949,6 @@
       <c r="T149" t="n">
         <v>5250</v>
       </c>
-      <c r="U149" t="inlineStr"/>
-      <c r="V149" t="inlineStr">
-        <is>
-          <t>Na</t>
-        </is>
-      </c>
-      <c r="W149" t="inlineStr">
-        <is>
-          <t>V-PE-50mM Na</t>
-        </is>
-      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -14047,17 +13033,6 @@
       <c r="T150" t="n">
         <v>7780</v>
       </c>
-      <c r="U150" t="inlineStr"/>
-      <c r="V150" t="inlineStr">
-        <is>
-          <t>Na</t>
-        </is>
-      </c>
-      <c r="W150" t="inlineStr">
-        <is>
-          <t>V-PE-10mM Na</t>
-        </is>
-      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -14142,21 +13117,6 @@
       <c r="T151" t="n">
         <v>17730</v>
       </c>
-      <c r="U151" t="inlineStr">
-        <is>
-          <t>Nature: river</t>
-        </is>
-      </c>
-      <c r="V151" t="inlineStr">
-        <is>
-          <t>Na</t>
-        </is>
-      </c>
-      <c r="W151" t="inlineStr">
-        <is>
-          <t>A-PE-10mM Na</t>
-        </is>
-      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -14241,17 +13201,6 @@
       <c r="T152" t="n">
         <v>4160</v>
       </c>
-      <c r="U152" t="inlineStr"/>
-      <c r="V152" t="inlineStr">
-        <is>
-          <t>Ca</t>
-        </is>
-      </c>
-      <c r="W152" t="inlineStr">
-        <is>
-          <t>V-PE-5mM Ca</t>
-        </is>
-      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -14336,17 +13285,6 @@
       <c r="T153" t="n">
         <v>6990</v>
       </c>
-      <c r="U153" t="inlineStr"/>
-      <c r="V153" t="inlineStr">
-        <is>
-          <t>Ca</t>
-        </is>
-      </c>
-      <c r="W153" t="inlineStr">
-        <is>
-          <t>V-PE-1mM Ca</t>
-        </is>
-      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -14431,21 +13369,6 @@
       <c r="T154" t="n">
         <v>8710</v>
       </c>
-      <c r="U154" t="inlineStr">
-        <is>
-          <t>Nature: river</t>
-        </is>
-      </c>
-      <c r="V154" t="inlineStr">
-        <is>
-          <t>Ca</t>
-        </is>
-      </c>
-      <c r="W154" t="inlineStr">
-        <is>
-          <t>A-PE-5mM Ca</t>
-        </is>
-      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -14530,13 +13453,6 @@
       <c r="T155" t="n">
         <v>536</v>
       </c>
-      <c r="U155" t="inlineStr"/>
-      <c r="V155" t="inlineStr"/>
-      <c r="W155" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -14621,13 +13537,6 @@
       <c r="T156" t="n">
         <v>670</v>
       </c>
-      <c r="U156" t="inlineStr"/>
-      <c r="V156" t="inlineStr"/>
-      <c r="W156" t="inlineStr">
-        <is>
-          <t>PLA</t>
-        </is>
-      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -14712,17 +13621,6 @@
       <c r="T157" t="n">
         <v>821</v>
       </c>
-      <c r="U157" t="inlineStr">
-        <is>
-          <t>Lab: UV/O3</t>
-        </is>
-      </c>
-      <c r="V157" t="inlineStr"/>
-      <c r="W157" t="inlineStr">
-        <is>
-          <t>APE</t>
-        </is>
-      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -14807,17 +13705,6 @@
       <c r="T158" t="n">
         <v>977</v>
       </c>
-      <c r="U158" t="inlineStr">
-        <is>
-          <t>Lab: UV/O3</t>
-        </is>
-      </c>
-      <c r="V158" t="inlineStr"/>
-      <c r="W158" t="inlineStr">
-        <is>
-          <t>APLA</t>
-        </is>
-      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -14900,13 +13787,6 @@
       <c r="T159" t="n">
         <v>78.73599999999999</v>
       </c>
-      <c r="U159" t="inlineStr"/>
-      <c r="V159" t="inlineStr"/>
-      <c r="W159" t="inlineStr">
-        <is>
-          <t>48 microm</t>
-        </is>
-      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -14989,13 +13869,6 @@
       <c r="T160" t="n">
         <v>39.9896</v>
       </c>
-      <c r="U160" t="inlineStr"/>
-      <c r="V160" t="inlineStr"/>
-      <c r="W160" t="inlineStr">
-        <is>
-          <t>125 microm</t>
-        </is>
-      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -15078,13 +13951,6 @@
       <c r="T161" t="n">
         <v>30.2512</v>
       </c>
-      <c r="U161" t="inlineStr"/>
-      <c r="V161" t="inlineStr"/>
-      <c r="W161" t="inlineStr">
-        <is>
-          <t>500 microm</t>
-        </is>
-      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -15167,13 +14033,6 @@
       <c r="T162" t="n">
         <v>16.1495</v>
       </c>
-      <c r="U162" t="inlineStr"/>
-      <c r="V162" t="inlineStr"/>
-      <c r="W162" t="inlineStr">
-        <is>
-          <t>Pb(II) = 0</t>
-        </is>
-      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -15256,17 +14115,6 @@
       <c r="T163" t="n">
         <v>14.4756</v>
       </c>
-      <c r="U163" t="inlineStr"/>
-      <c r="V163" t="inlineStr">
-        <is>
-          <t>Pb</t>
-        </is>
-      </c>
-      <c r="W163" t="inlineStr">
-        <is>
-          <t>Pb(II) = 0.005 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -15349,17 +14197,6 @@
       <c r="T164" t="n">
         <v>13.1719</v>
       </c>
-      <c r="U164" t="inlineStr"/>
-      <c r="V164" t="inlineStr">
-        <is>
-          <t>Pb</t>
-        </is>
-      </c>
-      <c r="W164" t="inlineStr">
-        <is>
-          <t>Pb(II) = 0.01 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -15442,17 +14279,6 @@
       <c r="T165" t="n">
         <v>9.2151</v>
       </c>
-      <c r="U165" t="inlineStr"/>
-      <c r="V165" t="inlineStr">
-        <is>
-          <t>Pb</t>
-        </is>
-      </c>
-      <c r="W165" t="inlineStr">
-        <is>
-          <t>Pb(II) = 0.05 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -15535,17 +14361,6 @@
       <c r="T166" t="n">
         <v>7.8111</v>
       </c>
-      <c r="U166" t="inlineStr"/>
-      <c r="V166" t="inlineStr">
-        <is>
-          <t>Pb</t>
-        </is>
-      </c>
-      <c r="W166" t="inlineStr">
-        <is>
-          <t>Pb(II) = 0.1 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -15628,13 +14443,6 @@
       <c r="T167" t="n">
         <v>23.8335</v>
       </c>
-      <c r="U167" t="inlineStr"/>
-      <c r="V167" t="inlineStr"/>
-      <c r="W167" t="inlineStr">
-        <is>
-          <t>Cu(II) = 0</t>
-        </is>
-      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -15717,17 +14525,6 @@
       <c r="T168" t="n">
         <v>20.1289</v>
       </c>
-      <c r="U168" t="inlineStr"/>
-      <c r="V168" t="inlineStr">
-        <is>
-          <t>Cu</t>
-        </is>
-      </c>
-      <c r="W168" t="inlineStr">
-        <is>
-          <t>Cu(II) = 0.005 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -15810,17 +14607,6 @@
       <c r="T169" t="n">
         <v>19.0987</v>
       </c>
-      <c r="U169" t="inlineStr"/>
-      <c r="V169" t="inlineStr">
-        <is>
-          <t>Cu</t>
-        </is>
-      </c>
-      <c r="W169" t="inlineStr">
-        <is>
-          <t>Cu(II) = 0.01 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -15903,17 +14689,6 @@
       <c r="T170" t="n">
         <v>13.9557</v>
       </c>
-      <c r="U170" t="inlineStr"/>
-      <c r="V170" t="inlineStr">
-        <is>
-          <t>Cu</t>
-        </is>
-      </c>
-      <c r="W170" t="inlineStr">
-        <is>
-          <t>Cu(II) = 0.05 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -15996,17 +14771,6 @@
       <c r="T171" t="n">
         <v>11.7943</v>
       </c>
-      <c r="U171" t="inlineStr"/>
-      <c r="V171" t="inlineStr">
-        <is>
-          <t>Cu</t>
-        </is>
-      </c>
-      <c r="W171" t="inlineStr">
-        <is>
-          <t>Cu(II) = 0.1 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -16089,17 +14853,6 @@
       <c r="T172" t="n">
         <v>19.8878</v>
       </c>
-      <c r="U172" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V172" t="inlineStr"/>
-      <c r="W172" t="inlineStr">
-        <is>
-          <t>Pb(II) = 0</t>
-        </is>
-      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -16182,17 +14935,6 @@
       <c r="T173" t="n">
         <v>16.7497</v>
       </c>
-      <c r="U173" t="inlineStr"/>
-      <c r="V173" t="inlineStr">
-        <is>
-          <t>Pb</t>
-        </is>
-      </c>
-      <c r="W173" t="inlineStr">
-        <is>
-          <t>Pb(II) = 0.005 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -16275,17 +15017,6 @@
       <c r="T174" t="n">
         <v>15.2978</v>
       </c>
-      <c r="U174" t="inlineStr"/>
-      <c r="V174" t="inlineStr">
-        <is>
-          <t>Pb</t>
-        </is>
-      </c>
-      <c r="W174" t="inlineStr">
-        <is>
-          <t>Pb(II) = 0.01 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -16368,17 +15099,6 @@
       <c r="T175" t="n">
         <v>11.463</v>
       </c>
-      <c r="U175" t="inlineStr"/>
-      <c r="V175" t="inlineStr">
-        <is>
-          <t>Pb</t>
-        </is>
-      </c>
-      <c r="W175" t="inlineStr">
-        <is>
-          <t>Pb(II) = 0.05 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -16461,17 +15181,6 @@
       <c r="T176" t="n">
         <v>10.4185</v>
       </c>
-      <c r="U176" t="inlineStr"/>
-      <c r="V176" t="inlineStr">
-        <is>
-          <t>Pb</t>
-        </is>
-      </c>
-      <c r="W176" t="inlineStr">
-        <is>
-          <t>Pb(II) = 0.1 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -16554,13 +15263,6 @@
       <c r="T177" t="n">
         <v>26.6819</v>
       </c>
-      <c r="U177" t="inlineStr"/>
-      <c r="V177" t="inlineStr"/>
-      <c r="W177" t="inlineStr">
-        <is>
-          <t>Cu(II) = 0</t>
-        </is>
-      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -16643,17 +15345,6 @@
       <c r="T178" t="n">
         <v>22.4351</v>
       </c>
-      <c r="U178" t="inlineStr"/>
-      <c r="V178" t="inlineStr">
-        <is>
-          <t>Cu</t>
-        </is>
-      </c>
-      <c r="W178" t="inlineStr">
-        <is>
-          <t>Cu(II) = 0.005 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -16736,17 +15427,6 @@
       <c r="T179" t="n">
         <v>21.4646</v>
       </c>
-      <c r="U179" t="inlineStr"/>
-      <c r="V179" t="inlineStr">
-        <is>
-          <t>Cu</t>
-        </is>
-      </c>
-      <c r="W179" t="inlineStr">
-        <is>
-          <t>Cu(II) = 0.01 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -16829,17 +15509,6 @@
       <c r="T180" t="n">
         <v>15.8741</v>
       </c>
-      <c r="U180" t="inlineStr"/>
-      <c r="V180" t="inlineStr">
-        <is>
-          <t>Cu</t>
-        </is>
-      </c>
-      <c r="W180" t="inlineStr">
-        <is>
-          <t>Cu(II) = 0.05 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -16922,17 +15591,6 @@
       <c r="T181" t="n">
         <v>13.0727</v>
       </c>
-      <c r="U181" t="inlineStr"/>
-      <c r="V181" t="inlineStr">
-        <is>
-          <t>Cu</t>
-        </is>
-      </c>
-      <c r="W181" t="inlineStr">
-        <is>
-          <t>Cu(II) = 0.1 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -17015,17 +15673,6 @@
       <c r="T182" t="n">
         <v>31.4048</v>
       </c>
-      <c r="U182" t="inlineStr">
-        <is>
-          <t>Lab: wastewater, aeration</t>
-        </is>
-      </c>
-      <c r="V182" t="inlineStr"/>
-      <c r="W182" t="inlineStr">
-        <is>
-          <t>Pb(II) = 0</t>
-        </is>
-      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -17108,17 +15755,6 @@
       <c r="T183" t="n">
         <v>30.5924</v>
       </c>
-      <c r="U183" t="inlineStr"/>
-      <c r="V183" t="inlineStr">
-        <is>
-          <t>Pb</t>
-        </is>
-      </c>
-      <c r="W183" t="inlineStr">
-        <is>
-          <t>Pb(II) = 0.005 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -17201,17 +15837,6 @@
       <c r="T184" t="n">
         <v>29.3424</v>
       </c>
-      <c r="U184" t="inlineStr"/>
-      <c r="V184" t="inlineStr">
-        <is>
-          <t>Pb</t>
-        </is>
-      </c>
-      <c r="W184" t="inlineStr">
-        <is>
-          <t>Pb(II) = 0.01 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -17294,17 +15919,6 @@
       <c r="T185" t="n">
         <v>28.5197</v>
       </c>
-      <c r="U185" t="inlineStr"/>
-      <c r="V185" t="inlineStr">
-        <is>
-          <t>Pb</t>
-        </is>
-      </c>
-      <c r="W185" t="inlineStr">
-        <is>
-          <t>Pb(II) = 0.05 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -17387,17 +16001,6 @@
       <c r="T186" t="n">
         <v>28.3158</v>
       </c>
-      <c r="U186" t="inlineStr"/>
-      <c r="V186" t="inlineStr">
-        <is>
-          <t>Pb</t>
-        </is>
-      </c>
-      <c r="W186" t="inlineStr">
-        <is>
-          <t>Pb(II) = 0.1 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -17480,13 +16083,6 @@
       <c r="T187" t="n">
         <v>43.8846</v>
       </c>
-      <c r="U187" t="inlineStr"/>
-      <c r="V187" t="inlineStr"/>
-      <c r="W187" t="inlineStr">
-        <is>
-          <t>Cu(II) = 0</t>
-        </is>
-      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -17569,17 +16165,6 @@
       <c r="T188" t="n">
         <v>41.7861</v>
       </c>
-      <c r="U188" t="inlineStr"/>
-      <c r="V188" t="inlineStr">
-        <is>
-          <t>Cu</t>
-        </is>
-      </c>
-      <c r="W188" t="inlineStr">
-        <is>
-          <t>Cu(II) = 0.005 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -17662,17 +16247,6 @@
       <c r="T189" t="n">
         <v>38.3453</v>
       </c>
-      <c r="U189" t="inlineStr"/>
-      <c r="V189" t="inlineStr">
-        <is>
-          <t>Cu</t>
-        </is>
-      </c>
-      <c r="W189" t="inlineStr">
-        <is>
-          <t>Cu(II) = 0.01 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -17755,17 +16329,6 @@
       <c r="T190" t="n">
         <v>34.5489</v>
       </c>
-      <c r="U190" t="inlineStr"/>
-      <c r="V190" t="inlineStr">
-        <is>
-          <t>Cu</t>
-        </is>
-      </c>
-      <c r="W190" t="inlineStr">
-        <is>
-          <t>Cu(II) = 0.05 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -17848,17 +16411,6 @@
       <c r="T191" t="n">
         <v>25.2635</v>
       </c>
-      <c r="U191" t="inlineStr"/>
-      <c r="V191" t="inlineStr">
-        <is>
-          <t>Cu</t>
-        </is>
-      </c>
-      <c r="W191" t="inlineStr">
-        <is>
-          <t>Cu(II) = 0.1 mmol/L</t>
-        </is>
-      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -17945,9 +16497,6 @@
       <c r="T192" t="n">
         <v>9.5</v>
       </c>
-      <c r="U192" t="inlineStr"/>
-      <c r="V192" t="inlineStr"/>
-      <c r="W192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -18034,13 +16583,6 @@
       <c r="T193" t="n">
         <v>167.4</v>
       </c>
-      <c r="U193" t="inlineStr">
-        <is>
-          <t>Lab: Sulfur, anaerobiosis</t>
-        </is>
-      </c>
-      <c r="V193" t="inlineStr"/>
-      <c r="W193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -18127,9 +16669,6 @@
       <c r="T194" t="n">
         <v>6.6</v>
       </c>
-      <c r="U194" t="inlineStr"/>
-      <c r="V194" t="inlineStr"/>
-      <c r="W194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -18216,13 +16755,6 @@
       <c r="T195" t="n">
         <v>35.7</v>
       </c>
-      <c r="U195" t="inlineStr">
-        <is>
-          <t>Lab: Sulfur, anaerobiosis</t>
-        </is>
-      </c>
-      <c r="V195" t="inlineStr"/>
-      <c r="W195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -18309,9 +16841,6 @@
       <c r="T196" t="n">
         <v>4.9</v>
       </c>
-      <c r="U196" t="inlineStr"/>
-      <c r="V196" t="inlineStr"/>
-      <c r="W196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -18398,13 +16927,6 @@
       <c r="T197" t="n">
         <v>44.1</v>
       </c>
-      <c r="U197" t="inlineStr">
-        <is>
-          <t>Lab: Sulfur, anaerobiosis</t>
-        </is>
-      </c>
-      <c r="V197" t="inlineStr"/>
-      <c r="W197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -18491,9 +17013,6 @@
       <c r="T198" t="n">
         <v>6.9</v>
       </c>
-      <c r="U198" t="inlineStr"/>
-      <c r="V198" t="inlineStr"/>
-      <c r="W198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -18580,13 +17099,6 @@
       <c r="T199" t="n">
         <v>15.9</v>
       </c>
-      <c r="U199" t="inlineStr">
-        <is>
-          <t>Lab: Sulfur, anaerobiosis</t>
-        </is>
-      </c>
-      <c r="V199" t="inlineStr"/>
-      <c r="W199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -18673,9 +17185,6 @@
       <c r="T200" t="n">
         <v>6.8</v>
       </c>
-      <c r="U200" t="inlineStr"/>
-      <c r="V200" t="inlineStr"/>
-      <c r="W200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -18762,13 +17271,6 @@
       <c r="T201" t="n">
         <v>38.2</v>
       </c>
-      <c r="U201" t="inlineStr">
-        <is>
-          <t>Lab: Sulfur, anaerobiosis</t>
-        </is>
-      </c>
-      <c r="V201" t="inlineStr"/>
-      <c r="W201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -18855,9 +17357,6 @@
       <c r="T202" t="n">
         <v>16.7</v>
       </c>
-      <c r="U202" t="inlineStr"/>
-      <c r="V202" t="inlineStr"/>
-      <c r="W202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -18944,13 +17443,6 @@
       <c r="T203" t="n">
         <v>244.6</v>
       </c>
-      <c r="U203" t="inlineStr">
-        <is>
-          <t>Lab: Sulfur, anaerobiosis</t>
-        </is>
-      </c>
-      <c r="V203" t="inlineStr"/>
-      <c r="W203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -19035,9 +17527,6 @@
       <c r="T204" t="n">
         <v>1230</v>
       </c>
-      <c r="U204" t="inlineStr"/>
-      <c r="V204" t="inlineStr"/>
-      <c r="W204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -19117,13 +17606,6 @@
       </c>
       <c r="T205" t="n">
         <v>151.802</v>
-      </c>
-      <c r="U205" t="inlineStr"/>
-      <c r="V205" t="inlineStr"/>
-      <c r="W205" t="inlineStr">
-        <is>
-          <t>P-PLA</t>
-        </is>
       </c>
     </row>
     <row r="206">
@@ -19201,17 +17683,6 @@
       <c r="T206" t="n">
         <v>1045.67</v>
       </c>
-      <c r="U206" t="inlineStr">
-        <is>
-          <t>Lab: Wastewater</t>
-        </is>
-      </c>
-      <c r="V206" t="inlineStr"/>
-      <c r="W206" t="inlineStr">
-        <is>
-          <t>S-PLA</t>
-        </is>
-      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -19294,9 +17765,6 @@
       <c r="T207" t="n">
         <v>146</v>
       </c>
-      <c r="U207" t="inlineStr"/>
-      <c r="V207" t="inlineStr"/>
-      <c r="W207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -19379,9 +17847,6 @@
       <c r="T208" t="n">
         <v>136</v>
       </c>
-      <c r="U208" t="inlineStr"/>
-      <c r="V208" t="inlineStr"/>
-      <c r="W208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -19464,9 +17929,6 @@
       <c r="T209" t="n">
         <v>767</v>
       </c>
-      <c r="U209" t="inlineStr"/>
-      <c r="V209" t="inlineStr"/>
-      <c r="W209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -19549,9 +18011,6 @@
       <c r="T210" t="n">
         <v>4930</v>
       </c>
-      <c r="U210" t="inlineStr"/>
-      <c r="V210" t="inlineStr"/>
-      <c r="W210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -19634,9 +18093,6 @@
       <c r="T211" t="n">
         <v>4150</v>
       </c>
-      <c r="U211" t="inlineStr"/>
-      <c r="V211" t="inlineStr"/>
-      <c r="W211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -19719,9 +18175,6 @@
       <c r="T212" t="n">
         <v>4740</v>
       </c>
-      <c r="U212" t="inlineStr"/>
-      <c r="V212" t="inlineStr"/>
-      <c r="W212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -19806,13 +18259,6 @@
       <c r="T213" t="n">
         <v>162</v>
       </c>
-      <c r="U213" t="inlineStr"/>
-      <c r="V213" t="inlineStr"/>
-      <c r="W213" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -19897,17 +18343,6 @@
       <c r="T214" t="n">
         <v>219</v>
       </c>
-      <c r="U214" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V214" t="inlineStr"/>
-      <c r="W214" t="inlineStr">
-        <is>
-          <t>UVPS</t>
-        </is>
-      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -19992,17 +18427,6 @@
       <c r="T215" t="n">
         <v>274</v>
       </c>
-      <c r="U215" t="inlineStr">
-        <is>
-          <t>Lab: H2O2</t>
-        </is>
-      </c>
-      <c r="V215" t="inlineStr"/>
-      <c r="W215" t="inlineStr">
-        <is>
-          <t>HOPS</t>
-        </is>
-      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -20087,17 +18511,6 @@
       <c r="T216" t="n">
         <v>154</v>
       </c>
-      <c r="U216" t="inlineStr"/>
-      <c r="V216" t="inlineStr">
-        <is>
-          <t>tetracycline</t>
-        </is>
-      </c>
-      <c r="W216" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -20182,21 +18595,6 @@
       <c r="T217" t="n">
         <v>246</v>
       </c>
-      <c r="U217" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V217" t="inlineStr">
-        <is>
-          <t>tetracycline</t>
-        </is>
-      </c>
-      <c r="W217" t="inlineStr">
-        <is>
-          <t>UVPS</t>
-        </is>
-      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -20281,21 +18679,6 @@
       <c r="T218" t="n">
         <v>290</v>
       </c>
-      <c r="U218" t="inlineStr">
-        <is>
-          <t>Lab: H2O2</t>
-        </is>
-      </c>
-      <c r="V218" t="inlineStr">
-        <is>
-          <t>tetracycline</t>
-        </is>
-      </c>
-      <c r="W218" t="inlineStr">
-        <is>
-          <t>HOPS</t>
-        </is>
-      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -20380,13 +18763,6 @@
       <c r="T219" t="n">
         <v>197</v>
       </c>
-      <c r="U219" t="inlineStr"/>
-      <c r="V219" t="inlineStr"/>
-      <c r="W219" t="inlineStr">
-        <is>
-          <t>PET</t>
-        </is>
-      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -20471,17 +18847,6 @@
       <c r="T220" t="n">
         <v>252</v>
       </c>
-      <c r="U220" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V220" t="inlineStr"/>
-      <c r="W220" t="inlineStr">
-        <is>
-          <t>UVPET</t>
-        </is>
-      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -20566,17 +18931,6 @@
       <c r="T221" t="n">
         <v>379</v>
       </c>
-      <c r="U221" t="inlineStr">
-        <is>
-          <t>Lab: H2O2</t>
-        </is>
-      </c>
-      <c r="V221" t="inlineStr"/>
-      <c r="W221" t="inlineStr">
-        <is>
-          <t>HOPET</t>
-        </is>
-      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -20661,17 +19015,6 @@
       <c r="T222" t="n">
         <v>200</v>
       </c>
-      <c r="U222" t="inlineStr"/>
-      <c r="V222" t="inlineStr">
-        <is>
-          <t>tetracycline</t>
-        </is>
-      </c>
-      <c r="W222" t="inlineStr">
-        <is>
-          <t>PET</t>
-        </is>
-      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -20756,21 +19099,6 @@
       <c r="T223" t="n">
         <v>313</v>
       </c>
-      <c r="U223" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V223" t="inlineStr">
-        <is>
-          <t>tetracycline</t>
-        </is>
-      </c>
-      <c r="W223" t="inlineStr">
-        <is>
-          <t>UVPET</t>
-        </is>
-      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -20855,21 +19183,6 @@
       <c r="T224" t="n">
         <v>392</v>
       </c>
-      <c r="U224" t="inlineStr">
-        <is>
-          <t>Lab: H2O2</t>
-        </is>
-      </c>
-      <c r="V224" t="inlineStr">
-        <is>
-          <t>tetracycline</t>
-        </is>
-      </c>
-      <c r="W224" t="inlineStr">
-        <is>
-          <t>HOPET</t>
-        </is>
-      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -20952,13 +19265,6 @@
       <c r="T225" t="n">
         <v>3880</v>
       </c>
-      <c r="U225" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V225" t="inlineStr"/>
-      <c r="W225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -21041,13 +19347,6 @@
       <c r="T226" t="n">
         <v>7120</v>
       </c>
-      <c r="U226" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V226" t="inlineStr"/>
-      <c r="W226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -21130,13 +19429,6 @@
       <c r="T227" t="n">
         <v>10100</v>
       </c>
-      <c r="U227" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V227" t="inlineStr"/>
-      <c r="W227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -21219,13 +19511,6 @@
       <c r="T228" t="n">
         <v>11.01</v>
       </c>
-      <c r="U228" t="inlineStr"/>
-      <c r="V228" t="inlineStr"/>
-      <c r="W228" t="inlineStr">
-        <is>
-          <t>PPw (CK)</t>
-        </is>
-      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -21308,17 +19593,6 @@
       <c r="T229" t="n">
         <v>6.85</v>
       </c>
-      <c r="U229" t="inlineStr">
-        <is>
-          <t>Nature: air-sun</t>
-        </is>
-      </c>
-      <c r="V229" t="inlineStr"/>
-      <c r="W229" t="inlineStr">
-        <is>
-          <t>PPw-30d</t>
-        </is>
-      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -21401,17 +19675,6 @@
       <c r="T230" t="n">
         <v>2.73</v>
       </c>
-      <c r="U230" t="inlineStr">
-        <is>
-          <t>Nature: air-sun</t>
-        </is>
-      </c>
-      <c r="V230" t="inlineStr"/>
-      <c r="W230" t="inlineStr">
-        <is>
-          <t>PPw-60d</t>
-        </is>
-      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -21494,17 +19757,6 @@
       <c r="T231" t="n">
         <v>1.35</v>
       </c>
-      <c r="U231" t="inlineStr">
-        <is>
-          <t>Nature: air-sun</t>
-        </is>
-      </c>
-      <c r="V231" t="inlineStr"/>
-      <c r="W231" t="inlineStr">
-        <is>
-          <t>PPw-120d</t>
-        </is>
-      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -21587,17 +19839,6 @@
       <c r="T232" t="n">
         <v>2.19</v>
       </c>
-      <c r="U232" t="inlineStr">
-        <is>
-          <t>Nature: air-sun</t>
-        </is>
-      </c>
-      <c r="V232" t="inlineStr"/>
-      <c r="W232" t="inlineStr">
-        <is>
-          <t>PPw-250d</t>
-        </is>
-      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -21680,13 +19921,6 @@
       <c r="T233" t="n">
         <v>9</v>
       </c>
-      <c r="U233" t="inlineStr"/>
-      <c r="V233" t="inlineStr"/>
-      <c r="W233" t="inlineStr">
-        <is>
-          <t>PEf-CK</t>
-        </is>
-      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -21769,17 +20003,6 @@
       <c r="T234" t="n">
         <v>6.34</v>
       </c>
-      <c r="U234" t="inlineStr">
-        <is>
-          <t>Nature: air-sun</t>
-        </is>
-      </c>
-      <c r="V234" t="inlineStr"/>
-      <c r="W234" t="inlineStr">
-        <is>
-          <t>Pef-30d</t>
-        </is>
-      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -21862,17 +20085,6 @@
       <c r="T235" t="n">
         <v>5.46</v>
       </c>
-      <c r="U235" t="inlineStr">
-        <is>
-          <t>Nature: air-sun</t>
-        </is>
-      </c>
-      <c r="V235" t="inlineStr"/>
-      <c r="W235" t="inlineStr">
-        <is>
-          <t>Pef-60d</t>
-        </is>
-      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -21955,17 +20167,6 @@
       <c r="T236" t="n">
         <v>2.26</v>
       </c>
-      <c r="U236" t="inlineStr">
-        <is>
-          <t>Nature: air-sun</t>
-        </is>
-      </c>
-      <c r="V236" t="inlineStr"/>
-      <c r="W236" t="inlineStr">
-        <is>
-          <t>Pef-90d</t>
-        </is>
-      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -22048,17 +20249,6 @@
       <c r="T237" t="n">
         <v>1.87</v>
       </c>
-      <c r="U237" t="inlineStr">
-        <is>
-          <t>Nature: air-sun</t>
-        </is>
-      </c>
-      <c r="V237" t="inlineStr"/>
-      <c r="W237" t="inlineStr">
-        <is>
-          <t>Pef-180d</t>
-        </is>
-      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -22141,17 +20331,6 @@
       <c r="T238" t="n">
         <v>1.05</v>
       </c>
-      <c r="U238" t="inlineStr">
-        <is>
-          <t>Nature: air-sun</t>
-        </is>
-      </c>
-      <c r="V238" t="inlineStr"/>
-      <c r="W238" t="inlineStr">
-        <is>
-          <t>Pef-250d</t>
-        </is>
-      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -22234,17 +20413,6 @@
       <c r="T239" t="n">
         <v>8840</v>
       </c>
-      <c r="U239" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V239" t="inlineStr"/>
-      <c r="W239" t="inlineStr">
-        <is>
-          <t>PS-CIP0</t>
-        </is>
-      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -22327,17 +20495,6 @@
       <c r="T240" t="n">
         <v>5010</v>
       </c>
-      <c r="U240" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V240" t="inlineStr"/>
-      <c r="W240" t="inlineStr">
-        <is>
-          <t>PS-CIP2</t>
-        </is>
-      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -22420,17 +20577,6 @@
       <c r="T241" t="n">
         <v>5360</v>
       </c>
-      <c r="U241" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V241" t="inlineStr"/>
-      <c r="W241" t="inlineStr">
-        <is>
-          <t>PVC-CIP0</t>
-        </is>
-      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -22513,17 +20659,6 @@
       <c r="T242" t="n">
         <v>7330</v>
       </c>
-      <c r="U242" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V242" t="inlineStr"/>
-      <c r="W242" t="inlineStr">
-        <is>
-          <t>PVC-CIP2</t>
-        </is>
-      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -22606,17 +20741,6 @@
       <c r="T243" t="n">
         <v>3080</v>
       </c>
-      <c r="U243" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V243" t="inlineStr"/>
-      <c r="W243" t="inlineStr">
-        <is>
-          <t>PS-CIP30</t>
-        </is>
-      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -22698,17 +20822,6 @@
       </c>
       <c r="T244" t="n">
         <v>2520</v>
-      </c>
-      <c r="U244" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V244" t="inlineStr"/>
-      <c r="W244" t="inlineStr">
-        <is>
-          <t>PVC-CIP30</t>
-        </is>
       </c>
     </row>
     <row r="245">
@@ -22790,13 +20903,6 @@
       <c r="T245" t="n">
         <v>11.8</v>
       </c>
-      <c r="U245" t="inlineStr">
-        <is>
-          <t>Lab+Nature: H202-Sunlight</t>
-        </is>
-      </c>
-      <c r="V245" t="inlineStr"/>
-      <c r="W245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -22877,13 +20983,6 @@
       <c r="T246" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="U246" t="inlineStr">
-        <is>
-          <t>Lab+Nature: H202-Sunlight</t>
-        </is>
-      </c>
-      <c r="V246" t="inlineStr"/>
-      <c r="W246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -22964,13 +21063,6 @@
       <c r="T247" t="n">
         <v>7.6</v>
       </c>
-      <c r="U247" t="inlineStr">
-        <is>
-          <t>Lab+Nature: H202-Sunlight</t>
-        </is>
-      </c>
-      <c r="V247" t="inlineStr"/>
-      <c r="W247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -23051,13 +21143,6 @@
       <c r="T248" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="U248" t="inlineStr">
-        <is>
-          <t>Lab+Nature: H202-Sunlight</t>
-        </is>
-      </c>
-      <c r="V248" t="inlineStr"/>
-      <c r="W248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -23138,13 +21223,6 @@
       <c r="T249" t="n">
         <v>11.4</v>
       </c>
-      <c r="U249" t="inlineStr">
-        <is>
-          <t>Lab+Nature: H202-Sunlight</t>
-        </is>
-      </c>
-      <c r="V249" t="inlineStr"/>
-      <c r="W249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -23229,9 +21307,6 @@
       <c r="T250" t="n">
         <v>1173</v>
       </c>
-      <c r="U250" t="inlineStr"/>
-      <c r="V250" t="inlineStr"/>
-      <c r="W250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -23316,13 +21391,6 @@
       <c r="T251" t="n">
         <v>1509</v>
       </c>
-      <c r="U251" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V251" t="inlineStr"/>
-      <c r="W251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -23407,9 +21475,6 @@
       <c r="T252" t="n">
         <v>894</v>
       </c>
-      <c r="U252" t="inlineStr"/>
-      <c r="V252" t="inlineStr"/>
-      <c r="W252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -23494,13 +21559,6 @@
       <c r="T253" t="n">
         <v>1210</v>
       </c>
-      <c r="U253" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V253" t="inlineStr"/>
-      <c r="W253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -23583,17 +21641,6 @@
       <c r="T254" t="n">
         <v>140.547</v>
       </c>
-      <c r="U254" t="inlineStr"/>
-      <c r="V254" t="inlineStr">
-        <is>
-          <t>P-PBAT</t>
-        </is>
-      </c>
-      <c r="W254" t="inlineStr">
-        <is>
-          <t>Pristin</t>
-        </is>
-      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -23676,21 +21723,6 @@
       <c r="T255" t="n">
         <v>172.065</v>
       </c>
-      <c r="U255" t="inlineStr">
-        <is>
-          <t>Lab: Wastewater</t>
-        </is>
-      </c>
-      <c r="V255" t="inlineStr">
-        <is>
-          <t>D-PBAT</t>
-        </is>
-      </c>
-      <c r="W255" t="inlineStr">
-        <is>
-          <t>Biodegrated</t>
-        </is>
-      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -23775,13 +21807,6 @@
       <c r="T256" t="n">
         <v>1910</v>
       </c>
-      <c r="U256" t="inlineStr"/>
-      <c r="V256" t="inlineStr"/>
-      <c r="W256" t="inlineStr">
-        <is>
-          <t>V-VPC+Pb</t>
-        </is>
-      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -23866,17 +21891,6 @@
       <c r="T257" t="n">
         <v>2630</v>
       </c>
-      <c r="U257" t="inlineStr"/>
-      <c r="V257" t="inlineStr">
-        <is>
-          <t>HA</t>
-        </is>
-      </c>
-      <c r="W257" t="inlineStr">
-        <is>
-          <t>V-VPC+Pb+5mg/L HA</t>
-        </is>
-      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -23961,17 +21975,6 @@
       <c r="T258" t="n">
         <v>3450</v>
       </c>
-      <c r="U258" t="inlineStr"/>
-      <c r="V258" t="inlineStr">
-        <is>
-          <t>HA</t>
-        </is>
-      </c>
-      <c r="W258" t="inlineStr">
-        <is>
-          <t>V-VPC+Pb+10mg/L HA</t>
-        </is>
-      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -24056,17 +22059,6 @@
       <c r="T259" t="n">
         <v>4040</v>
       </c>
-      <c r="U259" t="inlineStr"/>
-      <c r="V259" t="inlineStr">
-        <is>
-          <t>HA</t>
-        </is>
-      </c>
-      <c r="W259" t="inlineStr">
-        <is>
-          <t>V-VPC+Pb+15mg/L HA</t>
-        </is>
-      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -24151,21 +22143,6 @@
       <c r="T260" t="n">
         <v>4570</v>
       </c>
-      <c r="U260" t="inlineStr">
-        <is>
-          <t>Lab: Wastewater</t>
-        </is>
-      </c>
-      <c r="V260" t="inlineStr">
-        <is>
-          <t>HA</t>
-        </is>
-      </c>
-      <c r="W260" t="inlineStr">
-        <is>
-          <t>Bio-PVC-Pb</t>
-        </is>
-      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -24250,21 +22227,6 @@
       <c r="T261" t="n">
         <v>4420</v>
       </c>
-      <c r="U261" t="inlineStr">
-        <is>
-          <t>Lab: Wastewater</t>
-        </is>
-      </c>
-      <c r="V261" t="inlineStr">
-        <is>
-          <t>HA</t>
-        </is>
-      </c>
-      <c r="W261" t="inlineStr">
-        <is>
-          <t>Bio-PVC-Pb+5mg/L HA</t>
-        </is>
-      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -24349,21 +22311,6 @@
       <c r="T262" t="n">
         <v>4040</v>
       </c>
-      <c r="U262" t="inlineStr">
-        <is>
-          <t>Lab: Wastewater</t>
-        </is>
-      </c>
-      <c r="V262" t="inlineStr">
-        <is>
-          <t>HA</t>
-        </is>
-      </c>
-      <c r="W262" t="inlineStr">
-        <is>
-          <t>Bio-PVC-Pb+10mg/L HA</t>
-        </is>
-      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -24448,21 +22395,6 @@
       <c r="T263" t="n">
         <v>3440</v>
       </c>
-      <c r="U263" t="inlineStr">
-        <is>
-          <t>Lab: Wastewater</t>
-        </is>
-      </c>
-      <c r="V263" t="inlineStr">
-        <is>
-          <t>HA</t>
-        </is>
-      </c>
-      <c r="W263" t="inlineStr">
-        <is>
-          <t>Bio-PVC-Pb+15mg/L HA</t>
-        </is>
-      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -24547,13 +22479,6 @@
       <c r="T264" t="n">
         <v>889.54</v>
       </c>
-      <c r="U264" t="inlineStr"/>
-      <c r="V264" t="inlineStr"/>
-      <c r="W264" t="inlineStr">
-        <is>
-          <t>RPLA</t>
-        </is>
-      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -24638,17 +22563,6 @@
       <c r="T265" t="n">
         <v>1087.81</v>
       </c>
-      <c r="U265" t="inlineStr">
-        <is>
-          <t>Lab: sludge-hydrothermal treatment</t>
-        </is>
-      </c>
-      <c r="V265" t="inlineStr"/>
-      <c r="W265" t="inlineStr">
-        <is>
-          <t>PLA-110</t>
-        </is>
-      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -24733,17 +22647,6 @@
       <c r="T266" t="n">
         <v>1453.54</v>
       </c>
-      <c r="U266" t="inlineStr">
-        <is>
-          <t>Lab: sludge-hydrothermal treatment</t>
-        </is>
-      </c>
-      <c r="V266" t="inlineStr"/>
-      <c r="W266" t="inlineStr">
-        <is>
-          <t>PLA-120</t>
-        </is>
-      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -24828,17 +22731,6 @@
       <c r="T267" t="n">
         <v>1728.71</v>
       </c>
-      <c r="U267" t="inlineStr">
-        <is>
-          <t>Lab: sludge-hydrothermal treatment</t>
-        </is>
-      </c>
-      <c r="V267" t="inlineStr"/>
-      <c r="W267" t="inlineStr">
-        <is>
-          <t>PLA-130</t>
-        </is>
-      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -24923,17 +22815,6 @@
       <c r="T268" t="n">
         <v>2089.02</v>
       </c>
-      <c r="U268" t="inlineStr">
-        <is>
-          <t>Lab: sludge-hydrothermal treatment</t>
-        </is>
-      </c>
-      <c r="V268" t="inlineStr"/>
-      <c r="W268" t="inlineStr">
-        <is>
-          <t>PLA-140</t>
-        </is>
-      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -25018,13 +22899,6 @@
       <c r="T269" t="n">
         <v>6085</v>
       </c>
-      <c r="U269" t="inlineStr"/>
-      <c r="V269" t="inlineStr"/>
-      <c r="W269" t="inlineStr">
-        <is>
-          <t>PLA</t>
-        </is>
-      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -25109,17 +22983,6 @@
       <c r="T270" t="n">
         <v>7132</v>
       </c>
-      <c r="U270" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V270" t="inlineStr"/>
-      <c r="W270" t="inlineStr">
-        <is>
-          <t>aged-PLA</t>
-        </is>
-      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -25204,13 +23067,6 @@
       <c r="T271" t="n">
         <v>365</v>
       </c>
-      <c r="U271" t="inlineStr"/>
-      <c r="V271" t="inlineStr"/>
-      <c r="W271" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -25295,17 +23151,6 @@
       <c r="T272" t="n">
         <v>489</v>
       </c>
-      <c r="U272" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V272" t="inlineStr"/>
-      <c r="W272" t="inlineStr">
-        <is>
-          <t>aged-PLA</t>
-        </is>
-      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -25388,13 +23233,6 @@
       <c r="T273" t="n">
         <v>2.23</v>
       </c>
-      <c r="U273" t="inlineStr"/>
-      <c r="V273" t="inlineStr"/>
-      <c r="W273" t="inlineStr">
-        <is>
-          <t>P-PS</t>
-        </is>
-      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -25477,13 +23315,6 @@
       <c r="T274" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="U274" t="inlineStr"/>
-      <c r="V274" t="inlineStr"/>
-      <c r="W274" t="inlineStr">
-        <is>
-          <t>P-PE</t>
-        </is>
-      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -25566,13 +23397,6 @@
       <c r="T275" t="n">
         <v>12.54</v>
       </c>
-      <c r="U275" t="inlineStr"/>
-      <c r="V275" t="inlineStr"/>
-      <c r="W275" t="inlineStr">
-        <is>
-          <t>P-PLA</t>
-        </is>
-      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -25655,17 +23479,6 @@
       <c r="T276" t="n">
         <v>15.61</v>
       </c>
-      <c r="U276" t="inlineStr">
-        <is>
-          <t>Lab: O3 water</t>
-        </is>
-      </c>
-      <c r="V276" t="inlineStr"/>
-      <c r="W276" t="inlineStr">
-        <is>
-          <t>A-PS</t>
-        </is>
-      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -25748,17 +23561,6 @@
       <c r="T277" t="n">
         <v>22.23</v>
       </c>
-      <c r="U277" t="inlineStr">
-        <is>
-          <t>Lab: O3 water</t>
-        </is>
-      </c>
-      <c r="V277" t="inlineStr"/>
-      <c r="W277" t="inlineStr">
-        <is>
-          <t>A-PE</t>
-        </is>
-      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -25841,17 +23643,6 @@
       <c r="T278" t="n">
         <v>27.51</v>
       </c>
-      <c r="U278" t="inlineStr">
-        <is>
-          <t>Lab: O3 water</t>
-        </is>
-      </c>
-      <c r="V278" t="inlineStr"/>
-      <c r="W278" t="inlineStr">
-        <is>
-          <t>A-PLA</t>
-        </is>
-      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -25936,9 +23727,6 @@
       <c r="T279" t="n">
         <v>964</v>
       </c>
-      <c r="U279" t="inlineStr"/>
-      <c r="V279" t="inlineStr"/>
-      <c r="W279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -26023,13 +23811,6 @@
       <c r="T280" t="n">
         <v>1415</v>
       </c>
-      <c r="U280" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V280" t="inlineStr"/>
-      <c r="W280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -26114,9 +23895,6 @@
       <c r="T281" t="n">
         <v>951</v>
       </c>
-      <c r="U281" t="inlineStr"/>
-      <c r="V281" t="inlineStr"/>
-      <c r="W281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -26201,13 +23979,6 @@
       <c r="T282" t="n">
         <v>1398</v>
       </c>
-      <c r="U282" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V282" t="inlineStr"/>
-      <c r="W282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -26290,9 +24061,6 @@
       <c r="T283" t="n">
         <v>1997</v>
       </c>
-      <c r="U283" t="inlineStr"/>
-      <c r="V283" t="inlineStr"/>
-      <c r="W283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -26375,13 +24143,6 @@
       <c r="T284" t="n">
         <v>2192</v>
       </c>
-      <c r="U284" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V284" t="inlineStr"/>
-      <c r="W284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -26464,9 +24225,6 @@
       <c r="T285" t="n">
         <v>941</v>
       </c>
-      <c r="U285" t="inlineStr"/>
-      <c r="V285" t="inlineStr"/>
-      <c r="W285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -26549,13 +24307,6 @@
       <c r="T286" t="n">
         <v>1103</v>
       </c>
-      <c r="U286" t="inlineStr">
-        <is>
-          <t>Lab: UV</t>
-        </is>
-      </c>
-      <c r="V286" t="inlineStr"/>
-      <c r="W286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -26640,13 +24391,6 @@
       <c r="T287" t="n">
         <v>5167</v>
       </c>
-      <c r="U287" t="inlineStr"/>
-      <c r="V287" t="inlineStr"/>
-      <c r="W287" t="inlineStr">
-        <is>
-          <t>Ppa: 500 and 1000 μm</t>
-        </is>
-      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -26731,13 +24475,6 @@
       <c r="T288" t="n">
         <v>1805</v>
       </c>
-      <c r="U288" t="inlineStr"/>
-      <c r="V288" t="inlineStr"/>
-      <c r="W288" t="inlineStr">
-        <is>
-          <t>PPb: 250–500 μm</t>
-        </is>
-      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -26822,13 +24559,6 @@
       <c r="T289" t="n">
         <v>4494</v>
       </c>
-      <c r="U289" t="inlineStr"/>
-      <c r="V289" t="inlineStr"/>
-      <c r="W289" t="inlineStr">
-        <is>
-          <t>Aged PPb</t>
-        </is>
-      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -26913,13 +24643,6 @@
       <c r="T290" t="n">
         <v>4115</v>
       </c>
-      <c r="U290" t="inlineStr"/>
-      <c r="V290" t="inlineStr"/>
-      <c r="W290" t="inlineStr">
-        <is>
-          <t>PSa: 500 and 1000 μm</t>
-        </is>
-      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -27004,13 +24727,6 @@
       <c r="T291" t="n">
         <v>3814</v>
       </c>
-      <c r="U291" t="inlineStr"/>
-      <c r="V291" t="inlineStr"/>
-      <c r="W291" t="inlineStr">
-        <is>
-          <t>PSb: 250–500 μm</t>
-        </is>
-      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -27095,13 +24811,6 @@
       <c r="T292" t="n">
         <v>4445</v>
       </c>
-      <c r="U292" t="inlineStr"/>
-      <c r="V292" t="inlineStr"/>
-      <c r="W292" t="inlineStr">
-        <is>
-          <t>Aged PSb</t>
-        </is>
-      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -27186,13 +24895,6 @@
       <c r="T293" t="n">
         <v>7742</v>
       </c>
-      <c r="U293" t="inlineStr"/>
-      <c r="V293" t="inlineStr"/>
-      <c r="W293" t="inlineStr">
-        <is>
-          <t>Ppa: 500 and 1000 μm</t>
-        </is>
-      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -27277,13 +24979,6 @@
       <c r="T294" t="n">
         <v>5838</v>
       </c>
-      <c r="U294" t="inlineStr"/>
-      <c r="V294" t="inlineStr"/>
-      <c r="W294" t="inlineStr">
-        <is>
-          <t>PPb: 250–500 μm</t>
-        </is>
-      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -27368,13 +25063,6 @@
       <c r="T295" t="n">
         <v>9405</v>
       </c>
-      <c r="U295" t="inlineStr"/>
-      <c r="V295" t="inlineStr"/>
-      <c r="W295" t="inlineStr">
-        <is>
-          <t>Aged PPb</t>
-        </is>
-      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -27459,13 +25147,6 @@
       <c r="T296" t="n">
         <v>10979</v>
       </c>
-      <c r="U296" t="inlineStr"/>
-      <c r="V296" t="inlineStr"/>
-      <c r="W296" t="inlineStr">
-        <is>
-          <t>PSa: 500 and 1000 μm</t>
-        </is>
-      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -27550,13 +25231,6 @@
       <c r="T297" t="n">
         <v>10414</v>
       </c>
-      <c r="U297" t="inlineStr"/>
-      <c r="V297" t="inlineStr"/>
-      <c r="W297" t="inlineStr">
-        <is>
-          <t>PSb: 250–500 μm</t>
-        </is>
-      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -27640,13 +25314,6 @@
       </c>
       <c r="T298" t="n">
         <v>9263</v>
-      </c>
-      <c r="U298" t="inlineStr"/>
-      <c r="V298" t="inlineStr"/>
-      <c r="W298" t="inlineStr">
-        <is>
-          <t>Aged PSb</t>
-        </is>
       </c>
     </row>
     <row r="299">
@@ -27728,9 +25395,6 @@
       <c r="T299" t="n">
         <v>3690</v>
       </c>
-      <c r="U299" t="inlineStr"/>
-      <c r="V299" t="inlineStr"/>
-      <c r="W299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -27812,13 +25476,6 @@
       </c>
       <c r="T300" t="n">
         <v>4680</v>
-      </c>
-      <c r="U300" t="inlineStr"/>
-      <c r="V300" t="inlineStr"/>
-      <c r="W300" t="inlineStr">
-        <is>
-          <t>V-PPT</t>
-        </is>
       </c>
     </row>
     <row r="301">
@@ -27896,13 +25553,6 @@
       <c r="T301" t="n">
         <v>4120</v>
       </c>
-      <c r="U301" t="inlineStr"/>
-      <c r="V301" t="inlineStr"/>
-      <c r="W301" t="inlineStr">
-        <is>
-          <t>V-PPT</t>
-        </is>
-      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -27985,17 +25635,6 @@
       <c r="T302" t="n">
         <v>8990</v>
       </c>
-      <c r="U302" t="inlineStr">
-        <is>
-          <t>Lab: (biofilm) real wastewater</t>
-        </is>
-      </c>
-      <c r="V302" t="inlineStr"/>
-      <c r="W302" t="inlineStr">
-        <is>
-          <t>B-PPT</t>
-        </is>
-      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -28078,17 +25717,6 @@
       <c r="T303" t="n">
         <v>7180</v>
       </c>
-      <c r="U303" t="inlineStr">
-        <is>
-          <t>Lab: (biofilm) real wastewater</t>
-        </is>
-      </c>
-      <c r="V303" t="inlineStr"/>
-      <c r="W303" t="inlineStr">
-        <is>
-          <t>B-PPT</t>
-        </is>
-      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -28171,13 +25799,6 @@
       <c r="T304" t="n">
         <v>1000</v>
       </c>
-      <c r="U304" t="inlineStr"/>
-      <c r="V304" t="inlineStr"/>
-      <c r="W304" t="inlineStr">
-        <is>
-          <t>D-PPT</t>
-        </is>
-      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -28260,17 +25881,6 @@
       <c r="T305" t="n">
         <v>1200</v>
       </c>
-      <c r="U305" t="inlineStr">
-        <is>
-          <t>Lab: biodegraded MP</t>
-        </is>
-      </c>
-      <c r="V305" t="inlineStr"/>
-      <c r="W305" t="inlineStr">
-        <is>
-          <t>D-PPT</t>
-        </is>
-      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -28353,17 +25963,6 @@
       <c r="T306" t="n">
         <v>88</v>
       </c>
-      <c r="U306" t="inlineStr">
-        <is>
-          <t>Lab: biodegraded MP</t>
-        </is>
-      </c>
-      <c r="V306" t="inlineStr"/>
-      <c r="W306" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -28446,17 +26045,6 @@
       <c r="T307" t="n">
         <v>964</v>
       </c>
-      <c r="U307" t="inlineStr">
-        <is>
-          <t>Lab: distilled-water</t>
-        </is>
-      </c>
-      <c r="V307" t="inlineStr"/>
-      <c r="W307" t="inlineStr">
-        <is>
-          <t>PA-D</t>
-        </is>
-      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -28539,17 +26127,6 @@
       <c r="T308" t="n">
         <v>580</v>
       </c>
-      <c r="U308" t="inlineStr">
-        <is>
-          <t>Lab: tap-water</t>
-        </is>
-      </c>
-      <c r="V308" t="inlineStr"/>
-      <c r="W308" t="inlineStr">
-        <is>
-          <t>PA-T</t>
-        </is>
-      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -28632,17 +26209,6 @@
       <c r="T309" t="n">
         <v>282</v>
       </c>
-      <c r="U309" t="inlineStr">
-        <is>
-          <t>Lab: surface water</t>
-        </is>
-      </c>
-      <c r="V309" t="inlineStr"/>
-      <c r="W309" t="inlineStr">
-        <is>
-          <t>PA-S</t>
-        </is>
-      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -28725,17 +26291,6 @@
       <c r="T310" t="n">
         <v>1296</v>
       </c>
-      <c r="U310" t="inlineStr">
-        <is>
-          <t>Lab: wastewater</t>
-        </is>
-      </c>
-      <c r="V310" t="inlineStr"/>
-      <c r="W310" t="inlineStr">
-        <is>
-          <t>PA-W</t>
-        </is>
-      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -28818,13 +26373,6 @@
       <c r="T311" t="n">
         <v>1443</v>
       </c>
-      <c r="U311" t="inlineStr"/>
-      <c r="V311" t="inlineStr"/>
-      <c r="W311" t="inlineStr">
-        <is>
-          <t>PLA</t>
-        </is>
-      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -28907,17 +26455,6 @@
       <c r="T312" t="n">
         <v>2318</v>
       </c>
-      <c r="U312" t="inlineStr">
-        <is>
-          <t>Lab: distilled-water</t>
-        </is>
-      </c>
-      <c r="V312" t="inlineStr"/>
-      <c r="W312" t="inlineStr">
-        <is>
-          <t>PLA-D</t>
-        </is>
-      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -29000,17 +26537,6 @@
       <c r="T313" t="n">
         <v>1158</v>
       </c>
-      <c r="U313" t="inlineStr">
-        <is>
-          <t>Lab: tap-water</t>
-        </is>
-      </c>
-      <c r="V313" t="inlineStr"/>
-      <c r="W313" t="inlineStr">
-        <is>
-          <t>PLA-T</t>
-        </is>
-      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -29093,17 +26619,6 @@
       <c r="T314" t="n">
         <v>1207</v>
       </c>
-      <c r="U314" t="inlineStr">
-        <is>
-          <t>Lab: surface water</t>
-        </is>
-      </c>
-      <c r="V314" t="inlineStr"/>
-      <c r="W314" t="inlineStr">
-        <is>
-          <t>PLA-S</t>
-        </is>
-      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -29186,17 +26701,6 @@
       <c r="T315" t="n">
         <v>504</v>
       </c>
-      <c r="U315" t="inlineStr">
-        <is>
-          <t>Lab: wastewater</t>
-        </is>
-      </c>
-      <c r="V315" t="inlineStr"/>
-      <c r="W315" t="inlineStr">
-        <is>
-          <t>PLAW</t>
-        </is>
-      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -29279,9 +26783,6 @@
       <c r="T316" t="n">
         <v>2997</v>
       </c>
-      <c r="U316" t="inlineStr"/>
-      <c r="V316" t="inlineStr"/>
-      <c r="W316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -29364,9 +26865,6 @@
       <c r="T317" t="n">
         <v>2606</v>
       </c>
-      <c r="U317" t="inlineStr"/>
-      <c r="V317" t="inlineStr"/>
-      <c r="W317" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>